<commit_message>
GCV lambda selection: imaginary inversion + Re+Im cross-validation in all workflows
</commit_message>
<xml_diff>
--- a/lcurve_s2422_result.xlsx
+++ b/lcurve_s2422_result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mitra\Downloads\matlab analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2147E418-E3EA-4A4E-9A26-2D429F24F3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2671BE8D-7E05-4F17-B3A0-1099B00A2970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7A174AC2-1936-4A12-B49E-0DE59B899096}"/>
   </bookViews>
@@ -457,19 +457,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>9.9999999999999995E-7</v>
+        <v>1E-4</v>
       </c>
       <c r="B2">
-        <v>3128.3083870754726</v>
+        <v>3129.6683449588008</v>
       </c>
       <c r="C2">
-        <v>45381.023976821045</v>
+        <v>24485.805728993335</v>
       </c>
       <c r="D2">
-        <v>73.619528506977119</v>
+        <v>73.512123093201126</v>
       </c>
       <c r="E2">
-        <v>116.9078603620347</v>
+        <v>115.41256703449596</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -477,182 +477,182 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1.511775070615663E-6</v>
+        <v>2.7825594022071258E-4</v>
       </c>
       <c r="B3">
-        <v>3128.3202834610961</v>
+        <v>3130.365150779166</v>
       </c>
       <c r="C3">
-        <v>44038.659716659888</v>
+        <v>23380.215905376375</v>
       </c>
       <c r="D3">
-        <v>73.627367007278892</v>
+        <v>73.478527217347036</v>
       </c>
       <c r="E3">
-        <v>116.92920973684103</v>
+        <v>114.44540466946793</v>
       </c>
       <c r="F3">
-        <v>1.8503614478803539E-3</v>
+        <v>0.47692307193188305</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2.2854638641349884E-6</v>
+        <v>7.7426368268112698E-4</v>
       </c>
       <c r="B4">
-        <v>3128.3615683992962</v>
+        <v>3131.4238102412778</v>
       </c>
       <c r="C4">
-        <v>40887.213875447611</v>
+        <v>22776.969801767085</v>
       </c>
       <c r="D4">
-        <v>73.612104547259037</v>
+        <v>73.472040876661708</v>
       </c>
       <c r="E4">
-        <v>116.85266263223888</v>
+        <v>112.85386276686914</v>
       </c>
       <c r="F4">
-        <v>1.1263036948391824E-3</v>
+        <v>2.0138904887607074</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>3.4551072945922181E-6</v>
+        <v>2.1544346900318821E-3</v>
       </c>
       <c r="B5">
-        <v>3128.4202961878723</v>
+        <v>3134.2083558714071</v>
       </c>
       <c r="C5">
-        <v>37502.592653226973</v>
+        <v>22211.899247877638</v>
       </c>
       <c r="D5">
-        <v>73.602463129503136</v>
+        <v>74.148860690909672</v>
       </c>
       <c r="E5">
-        <v>116.77803887451013</v>
+        <v>110.16050857878501</v>
       </c>
       <c r="F5">
-        <v>2.106772579167505E-3</v>
+        <v>4.5223532371427115</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>5.2233450742668436E-6</v>
+        <v>5.9948425031894088E-3</v>
       </c>
       <c r="B6">
-        <v>3128.4706393693064</v>
+        <v>3143.3294455910241</v>
       </c>
       <c r="C6">
-        <v>35447.897870391374</v>
+        <v>21522.223039526285</v>
       </c>
       <c r="D6">
-        <v>73.591833327204881</v>
+        <v>77.302939217230275</v>
       </c>
       <c r="E6">
-        <v>116.71120869406069</v>
+        <v>105.78445140914532</v>
       </c>
       <c r="F6">
-        <v>4.4833230744291529E-3</v>
+        <v>9.5642748137857421</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7.8965228684997334E-6</v>
+        <v>1.6681005372000592E-2</v>
       </c>
       <c r="B7">
-        <v>3128.5304836710884</v>
+        <v>3167.8567917935361</v>
       </c>
       <c r="C7">
-        <v>33746.163600383261</v>
+        <v>20815.04895405575</v>
       </c>
       <c r="D7">
-        <v>73.596121835915</v>
+        <v>85.365518437822175</v>
       </c>
       <c r="E7">
-        <v>116.68640396095064</v>
+        <v>99.842582083054012</v>
       </c>
       <c r="F7">
-        <v>5.4971604109781214E-3</v>
+        <v>21.019369537471711</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1.1937766417144358E-5</v>
+        <v>4.6415888336127774E-2</v>
       </c>
       <c r="B8">
-        <v>3128.6501454992454</v>
+        <v>3221.5370632215058</v>
       </c>
       <c r="C8">
-        <v>31428.049524941289</v>
+        <v>20227.748478324491</v>
       </c>
       <c r="D8">
-        <v>73.579913460635439</v>
+        <v>98.993569145539198</v>
       </c>
       <c r="E8">
-        <v>116.54091144409746</v>
+        <v>93.320089406934898</v>
       </c>
       <c r="F8">
-        <v>5.1926959310138023E-3</v>
+        <v>25.8150545932901</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1.8047217668271701E-5</v>
+        <v>0.12915496650148839</v>
       </c>
       <c r="B9">
-        <v>3128.789241166497</v>
+        <v>3352.6578730744691</v>
       </c>
       <c r="C9">
-        <v>29468.762271707488</v>
+        <v>19696.740927174033</v>
       </c>
       <c r="D9">
-        <v>73.5654168105564</v>
+        <v>120.55660502742241</v>
       </c>
       <c r="E9">
-        <v>116.38544436991566</v>
+        <v>88.843546303730463</v>
       </c>
       <c r="F9">
-        <v>9.6454615405994811E-3</v>
+        <v>6.0093484491335953</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>2.7283333764867696E-5</v>
+        <v>0.35938136638046259</v>
       </c>
       <c r="B10">
-        <v>3128.9317468854738</v>
+        <v>3812.4917783406954</v>
       </c>
       <c r="C10">
-        <v>28063.784429500702</v>
+        <v>18966.659309118073</v>
       </c>
       <c r="D10">
-        <v>73.56394328125117</v>
+        <v>175.01316498934236</v>
       </c>
       <c r="E10">
-        <v>116.2732751812806</v>
+        <v>95.693180494416751</v>
       </c>
       <c r="F10">
-        <v>1.3141417716034418E-2</v>
+        <v>0.72687288692279417</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>4.1246263829013477E-5</v>
+        <v>1</v>
       </c>
       <c r="B11">
-        <v>3129.1744892847364</v>
+        <v>5391.7615748475891</v>
       </c>
       <c r="C11">
-        <v>26378.828023952454</v>
+        <v>17746.122560149131</v>
       </c>
       <c r="D11">
-        <v>73.536852205187643</v>
+        <v>305.12819679050654</v>
       </c>
       <c r="E11">
-        <v>115.97742356888654</v>
+        <v>145.79791326286286</v>
       </c>
       <c r="F11">
-        <v>1.9936929951257665E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1287,22 +1287,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>4.6415888336127822E-2</v>
+        <v>4.6415888336127774E-2</v>
       </c>
       <c r="B2">
-        <v>3221.537063221504</v>
+        <v>3221.5370632215058</v>
       </c>
       <c r="C2">
-        <v>20227.748478324502</v>
+        <v>20227.748478324491</v>
       </c>
       <c r="D2">
-        <v>98.993569145538942</v>
+        <v>98.993569145539198</v>
       </c>
       <c r="E2">
-        <v>93.320089406935438</v>
+        <v>93.320089406934898</v>
       </c>
       <c r="F2">
-        <v>29.242691031880312</v>
+        <v>25.8150545932901</v>
       </c>
     </row>
   </sheetData>

</xml_diff>